<commit_message>
fix: an Excel cell's type is read before the tokenizer's buffer can move under it — past the first 64 KB a shared string could read as its index — and a formula's text is entity-decoded once, so an & in it no longer fails the read
</commit_message>
<xml_diff>
--- a/src/connect/testdata/edge.xlsx
+++ b/src/connect/testdata/edge.xlsx
@@ -113,6 +113,10 @@
       <x:c r="F3" s="2">
         <x:v>0.1</x:v>
       </x:c>
+      <x:c r="G3" t="str">
+        <x:f>"Silva"&amp;" &amp; Filhos"</x:f>
+        <x:v>Silva &amp; Filhos_x000D_&amp;lt;</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">

</xml_diff>